<commit_message>
Fix Streamlit app imports and update watchlist outputs
</commit_message>
<xml_diff>
--- a/evaluation/results/watchlist_latest.xlsx
+++ b/evaluation/results/watchlist_latest.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,51 +425,51 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Stock</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Prediction</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Expected_Movement</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Confidence</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Confidence_Level</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Recommendation</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Last_Date</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Last_Close</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>XAI_Factors</t>
         </is>
@@ -466,32 +478,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>LT</t>
+          <t>HDFCBANK</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>-1.30%</t>
+          <t>+4.23%</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>58.0%</t>
+          <t>87.3%</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>AVOID</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -501,44 +513,44 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Rs.4079.95</t>
+          <t>Rs.795.45</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>📈 Market volatility is moderately pushing price UP | 📉 Daily price swing size is moderately pulling price DOWN | 📉 Market return this week is moderately pulling price DOWN | 📉 Momentum (overbought/oversold) is moderately pulling price DOWN | 📉 Price vs 20-day average is slightly pulling price DOWN</t>
+          <t>📈 Market volatility is strongly pushing price UP | 📈 Distance from 52-week high is strongly pushing price UP | 📈 Trend strength is moderately pushing price UP | 📉 Market return this week is moderately pulling price DOWN | 📈 Return on equity is moderately pushing price UP</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>TITAN</t>
+          <t>ITC</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>-1.30%</t>
+          <t>+4.21%</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>58.0%</t>
+          <t>87.1%</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>AVOID</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -548,12 +560,388 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Rs.4461.40</t>
+          <t>Rs.295.35</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>📈 Market volatility is moderately pushing price UP | 📉 Distance from 52-week high is moderately pulling price DOWN | 📈 Trend strength is moderately pushing price UP | 📉 Price-to-Earnings ratio is moderately pulling price DOWN | 📉 Market return this week is moderately pulling price DOWN</t>
+          <t>📈 Market volatility is strongly pushing price UP | 📈 Distance from 52-week high is strongly pushing price UP | 📈 Profit growth is moderately pushing price UP | 📈 Trend strength is moderately pushing price UP | 📈 Price vs 50-day average is moderately pushing price UP</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>INDUSINDBK</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>+3.96%</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>84.6%</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Rs.847.90</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>📈 Market volatility is strongly pushing price UP | 📈 Trend strength is moderately pushing price UP | 📈 Distance from 52-week high is moderately pushing price UP | 📈 Return on equity is moderately pushing price UP | 📉 Profit growth is moderately pulling price DOWN</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>SBIN</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>+3.94%</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>84.4%</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Rs.1052.53</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>📈 Market volatility is strongly pushing price UP | 📈 Distance from 52-week high is moderately pushing price UP | 📈 Price-to-Earnings ratio is moderately pushing price UP | 📈 Trend strength is moderately pushing price UP | 📉 Volatility vs history is moderately pulling price DOWN</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>RELIANCE</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>+3.69%</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>81.9%</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Rs.1343.30</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>📈 Market volatility is strongly pushing price UP | 📈 Distance from 52-week high is strongly pushing price UP | 📈 Return on equity is moderately pushing price UP | 📉 Market return this week is moderately pulling price DOWN | 📉 Market trend (20 days) is moderately pulling price DOWN</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>MARUTI</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>+3.47%</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>79.7%</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Rs.13076.00</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>📈 Market volatility is strongly pushing price UP | 📈 Distance from 52-week high is strongly pushing price UP | 📉 Market return this week is moderately pulling price DOWN | 📈 Sector return this week is moderately pushing price UP | 📈 Days since last news is moderately pushing price UP</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>GRASIM</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>+3.40%</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>79.0%</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Rs.2717.30</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>📈 Market volatility is strongly pushing price UP | 📈 Trend strength is moderately pushing price UP | 📈 Return on equity is moderately pushing price UP | 📈 Revenue growth is moderately pushing price UP | 📉 Market return this week is slightly pulling price DOWN</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>M&amp;M</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>+3.35%</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>78.5%</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Rs.3222.30</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>📈 Market volatility is strongly pushing price UP | 📈 Distance from 52-week high is moderately pushing price UP | 📈 Trend strength is moderately pushing price UP | 📉 Market return this week is moderately pulling price DOWN | 📈 Financials are outdated is moderately pushing price UP</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>HEROMOTOCO</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>+3.32%</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>78.2%</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Rs.5287.50</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>📈 Market volatility is strongly pushing price UP | 📈 Distance from 52-week high is strongly pushing price UP | 📉 Market return this week is moderately pulling price DOWN | 📉 Profit growth is moderately pulling price DOWN | 📈 Trend strength is moderately pushing price UP</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>COALINDIA</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>+3.20%</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>77.0%</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Rs.432.75</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>📈 Market volatility is strongly pushing price UP | 📈 Price-to-Earnings ratio is strongly pushing price UP | 📉 Trend strength is moderately pulling price DOWN | 📉 Market return this week is moderately pulling price DOWN | 📉 Return on equity is slightly pulling price DOWN</t>
         </is>
       </c>
     </row>

</xml_diff>